<commit_message>
Refresh corrected bank specimen deliverables after BOG and SCB parser fixes.
Re-export parsed comparisons and update the client zip with the 5M BOG credit and full SCB statement including first page and 540,206.03 closing balance.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/corrected-bank-specimens-for-user/13-bog/parsed-excel/BOG COCOBOD GHS ADV OPERATIONAL EXP ACCT(01102022-30092023) - parsed.xlsx
+++ b/corrected-bank-specimens-for-user/13-bog/parsed-excel/BOG COCOBOD GHS ADV OPERATIONAL EXP ACCT(01102022-30092023) - parsed.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G55"/>
+  <dimension ref="A1:G56"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -427,7 +427,7 @@
         <v>Exported</v>
       </c>
       <c r="B4" t="str">
-        <v>2026-07-08T16:17:01.679Z</v>
+        <v>2026-07-14T13:50:04.477Z</v>
       </c>
     </row>
     <row r="5">
@@ -435,7 +435,7 @@
         <v>Row count</v>
       </c>
       <c r="B5">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="6">
@@ -451,7 +451,7 @@
         <v>Sum credits / receipts</v>
       </c>
       <c r="B7">
-        <v>2000000</v>
+        <v>7000000</v>
       </c>
     </row>
     <row r="9">
@@ -493,6 +493,9 @@
       <c r="E10">
         <v>247742.86</v>
       </c>
+      <c r="G10">
+        <v>805982.66</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
@@ -510,6 +513,9 @@
       <c r="E11">
         <v>3775.1</v>
       </c>
+      <c r="G11">
+        <v>802207.56</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
@@ -527,6 +533,9 @@
       <c r="E12">
         <v>184813</v>
       </c>
+      <c r="G12">
+        <v>617394.56</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
@@ -544,6 +553,9 @@
       <c r="E13">
         <v>250623.71</v>
       </c>
+      <c r="G13">
+        <v>366770.85</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
@@ -682,6 +694,9 @@
       <c r="E20">
         <v>198204.05</v>
       </c>
+      <c r="G20">
+        <v>1396899.56</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
@@ -699,6 +714,9 @@
       <c r="E21">
         <v>176161.44</v>
       </c>
+      <c r="G21">
+        <v>1220738.12</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
@@ -716,6 +734,9 @@
       <c r="E22">
         <v>125149.44</v>
       </c>
+      <c r="G22">
+        <v>1095588.68</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
@@ -733,6 +754,9 @@
       <c r="E23">
         <v>39413.88</v>
       </c>
+      <c r="G23">
+        <v>1056174.8</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
@@ -750,6 +774,9 @@
       <c r="E24">
         <v>42169.92</v>
       </c>
+      <c r="G24">
+        <v>1014004.88</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
@@ -767,6 +794,9 @@
       <c r="E25">
         <v>123108.96</v>
       </c>
+      <c r="G25">
+        <v>890895.92</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
@@ -784,6 +814,9 @@
       <c r="E26">
         <v>82979.52</v>
       </c>
+      <c r="G26">
+        <v>807916.4</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
@@ -882,6 +915,9 @@
       <c r="E31">
         <v>136939.16</v>
       </c>
+      <c r="G31">
+        <v>553225.25</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
@@ -899,6 +935,9 @@
       <c r="E32">
         <v>331616</v>
       </c>
+      <c r="G32">
+        <v>221609.25</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
@@ -916,6 +955,9 @@
       <c r="E33">
         <v>68469.58</v>
       </c>
+      <c r="G33">
+        <v>153139.67</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
@@ -933,6 +975,9 @@
       <c r="E34">
         <v>6585.84</v>
       </c>
+      <c r="G34">
+        <v>146553.83</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
@@ -950,22 +995,28 @@
       <c r="E35">
         <v>95232.51</v>
       </c>
+      <c r="G35">
+        <v>51321.32</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>22/06/2023</v>
+        <v>09/06/2023</v>
       </c>
       <c r="B36" t="str">
-        <v>Cash Withdrawal WDR AKO-ABANG MABEL IFO SAMUEL SAKA BOATENG AND OTHERS</v>
+        <v>Transfer BANK OF GHANA TRSF PER DEC/FA/BOG/5/V.10/132 IRO PMT OF COCOA BEANS DD 08/06/2023</v>
       </c>
       <c r="C36" t="str">
-        <v>TT2317300400</v>
+        <v>FT2316074433</v>
       </c>
       <c r="D36" t="str">
-        <v>22/06/2023</v>
-      </c>
-      <c r="E36">
-        <v>142361.94</v>
+        <v>09/06/2023</v>
+      </c>
+      <c r="F36">
+        <v>5000000</v>
+      </c>
+      <c r="G36">
+        <v>5051321.32</v>
       </c>
     </row>
     <row r="37">
@@ -973,33 +1024,39 @@
         <v>22/06/2023</v>
       </c>
       <c r="B37" t="str">
-        <v>Cash Withdrawal WDR AKO-ABANG MABEL IFO REV.EDWIN AFARI AND OTHER</v>
+        <v>Cash Withdrawal WDR AKO-ABANG MABEL IFO SAMUEL SAKA BOATENG AND OTHERS</v>
       </c>
       <c r="C37" t="str">
-        <v>TT2317300473</v>
+        <v>TT2317300400</v>
       </c>
       <c r="D37" t="str">
         <v>22/06/2023</v>
       </c>
       <c r="E37">
-        <v>19787.76</v>
+        <v>142361.94</v>
+      </c>
+      <c r="G37">
+        <v>4908959.38</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>29/06/2023</v>
+        <v>22/06/2023</v>
       </c>
       <c r="B38" t="str">
-        <v>Cash Withdrawal WDR AKO-ABANG MABEL IFO EDWARD AMOAH ODAME</v>
+        <v>Cash Withdrawal WDR AKO-ABANG MABEL IFO REV.EDWIN AFARI AND OTHER</v>
       </c>
       <c r="C38" t="str">
-        <v>TT2318000477</v>
+        <v>TT2317300473</v>
       </c>
       <c r="D38" t="str">
-        <v>29/06/2023</v>
+        <v>22/06/2023</v>
       </c>
       <c r="E38">
-        <v>67119.52</v>
+        <v>19787.76</v>
+      </c>
+      <c r="G38">
+        <v>4889171.62</v>
       </c>
     </row>
     <row r="39">
@@ -1007,16 +1064,19 @@
         <v>29/06/2023</v>
       </c>
       <c r="B39" t="str">
-        <v>Cash Withdrawal WDR AKO-ABANG MABEL IFO DR.MOSES KWAME AIDOO</v>
+        <v>Cash Withdrawal WDR AKO-ABANG MABEL IFO EDWARD AMOAH ODAME</v>
       </c>
       <c r="C39" t="str">
-        <v>TT2318000471</v>
+        <v>TT2318000477</v>
       </c>
       <c r="D39" t="str">
         <v>29/06/2023</v>
       </c>
       <c r="E39">
-        <v>6601.92</v>
+        <v>67119.52</v>
+      </c>
+      <c r="G39">
+        <v>4822052.1</v>
       </c>
     </row>
     <row r="40">
@@ -1024,16 +1084,19 @@
         <v>29/06/2023</v>
       </c>
       <c r="B40" t="str">
-        <v>Cash Withdrawal WDR AKO-ABANG MABEL IFO KOFI TETTEH AND OTHERS</v>
+        <v>Cash Withdrawal WDR AKO-ABANG MABEL IFO DR.MOSES KWAME AIDOO</v>
       </c>
       <c r="C40" t="str">
-        <v>TT2318000532</v>
+        <v>TT2318000471</v>
       </c>
       <c r="D40" t="str">
         <v>29/06/2023</v>
       </c>
       <c r="E40">
-        <v>84445.9</v>
+        <v>6601.92</v>
+      </c>
+      <c r="G40">
+        <v>4815450.18</v>
       </c>
     </row>
     <row r="41">
@@ -1041,87 +1104,99 @@
         <v>29/06/2023</v>
       </c>
       <c r="B41" t="str">
-        <v>Cash Withdrawal WDR AKO-ABANG MABEL IFO ALBERT YEBOAH AND OTHERS</v>
+        <v>Cash Withdrawal WDR AKO-ABANG MABEL IFO KOFI TETTEH AND OTHERS</v>
       </c>
       <c r="C41" t="str">
-        <v>TT2318000543</v>
+        <v>TT2318000532</v>
       </c>
       <c r="D41" t="str">
         <v>29/06/2023</v>
       </c>
       <c r="E41">
-        <v>316068.94</v>
+        <v>84445.9</v>
+      </c>
+      <c r="G41">
+        <v>4731004.28</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>07/07/2023</v>
+        <v>29/06/2023</v>
       </c>
       <c r="B42" t="str">
-        <v>Cash Withdrawal WDR THERSON-COFIE FRANCES MAKU IFO RICHARD ADU-ACHEAMPONG</v>
+        <v>Cash Withdrawal WDR AKO-ABANG MABEL IFO ALBERT YEBOAH AND OTHERS</v>
       </c>
       <c r="C42" t="str">
-        <v>TT2318800503</v>
+        <v>TT2318000543</v>
       </c>
       <c r="D42" t="str">
-        <v>07/07/2023</v>
+        <v>29/06/2023</v>
       </c>
       <c r="E42">
-        <v>9905.31</v>
+        <v>316068.94</v>
+      </c>
+      <c r="G42">
+        <v>4414935.34</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>27/07/2023</v>
+        <v>07/07/2023</v>
       </c>
       <c r="B43" t="str">
-        <v>Cash Withdrawal WDR THERSON-COFIE FRANCIES MAKU IFO PAZ O. BOAKYE AND OTHERS</v>
+        <v>Cash Withdrawal WDR THERSON-COFIE FRANCES MAKU IFO RICHARD ADU-ACHEAMPONG</v>
       </c>
       <c r="C43" t="str">
-        <v>TT2320800610</v>
+        <v>TT2318800503</v>
       </c>
       <c r="D43" t="str">
-        <v>27/07/2023</v>
+        <v>07/07/2023</v>
       </c>
       <c r="E43">
-        <v>392982.6</v>
+        <v>9905.31</v>
+      </c>
+      <c r="G43">
+        <v>4405030.03</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>03/08/2023</v>
+        <v>27/07/2023</v>
       </c>
       <c r="B44" t="str">
-        <v>Cash Withdrawal WDR THERSON-COFIE FRANCES MAKU</v>
+        <v>Cash Withdrawal WDR THERSON-COFIE FRANCIES MAKU IFO PAZ O. BOAKYE AND OTHERS</v>
       </c>
       <c r="C44" t="str">
-        <v>TT2321500969</v>
+        <v>TT2320800610</v>
       </c>
       <c r="D44" t="str">
-        <v>03/08/2023</v>
+        <v>27/07/2023</v>
       </c>
       <c r="E44">
-        <v>80359.13</v>
+        <v>392982.6</v>
+      </c>
+      <c r="G44">
+        <v>4012047.43</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>10/08/2023</v>
+        <v>03/08/2023</v>
       </c>
       <c r="B45" t="str">
-        <v>Cash Withdrawal</v>
+        <v>Cash Withdrawal WDR THERSON-COFIE FRANCES MAKU</v>
       </c>
       <c r="C45" t="str">
-        <v>TT2322200348</v>
+        <v>TT2321500969</v>
       </c>
       <c r="D45" t="str">
-        <v>10/08/2023</v>
+        <v>03/08/2023</v>
       </c>
       <c r="E45">
-        <v>134296.38</v>
+        <v>80359.13</v>
       </c>
       <c r="G45">
-        <v>3797391.92</v>
+        <v>3931688.3</v>
       </c>
     </row>
     <row r="46">
@@ -1132,16 +1207,16 @@
         <v>Cash Withdrawal</v>
       </c>
       <c r="C46" t="str">
-        <v>TT2322200646</v>
+        <v>TT2322200348</v>
       </c>
       <c r="D46" t="str">
         <v>10/08/2023</v>
       </c>
       <c r="E46">
-        <v>201444.57</v>
+        <v>134296.38</v>
       </c>
       <c r="G46">
-        <v>3595947.35</v>
+        <v>3797391.92</v>
       </c>
     </row>
     <row r="47">
@@ -1152,36 +1227,36 @@
         <v>Cash Withdrawal</v>
       </c>
       <c r="C47" t="str">
-        <v>TT2322200664</v>
+        <v>TT2322200646</v>
       </c>
       <c r="D47" t="str">
         <v>10/08/2023</v>
       </c>
       <c r="E47">
-        <v>280438</v>
+        <v>201444.57</v>
       </c>
       <c r="G47">
-        <v>3315509.35</v>
+        <v>3595947.35</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>25/08/2023</v>
+        <v>10/08/2023</v>
       </c>
       <c r="B48" t="str">
         <v>Cash Withdrawal</v>
       </c>
       <c r="C48" t="str">
-        <v>TT2323700420</v>
+        <v>TT2322200664</v>
       </c>
       <c r="D48" t="str">
-        <v>25/08/2023</v>
+        <v>10/08/2023</v>
       </c>
       <c r="E48">
-        <v>118947.96</v>
+        <v>280438</v>
       </c>
       <c r="G48">
-        <v>3196561.39</v>
+        <v>3315509.35</v>
       </c>
     </row>
     <row r="49">
@@ -1192,71 +1267,77 @@
         <v>Cash Withdrawal</v>
       </c>
       <c r="C49" t="str">
-        <v>TT2323700437</v>
+        <v>TT2323700420</v>
       </c>
       <c r="D49" t="str">
         <v>25/08/2023</v>
       </c>
       <c r="E49">
-        <v>258236.42</v>
+        <v>118947.96</v>
       </c>
       <c r="G49">
-        <v>2938324.97</v>
+        <v>3196561.39</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
+        <v>25/08/2023</v>
+      </c>
+      <c r="B50" t="str">
+        <v>Cash Withdrawal</v>
+      </c>
+      <c r="C50" t="str">
+        <v>TT2323700437</v>
+      </c>
+      <c r="D50" t="str">
+        <v>25/08/2023</v>
+      </c>
+      <c r="E50">
+        <v>258236.42</v>
+      </c>
+      <c r="G50">
+        <v>2938324.97</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
         <v>29/08/2023</v>
       </c>
-      <c r="B50" t="str">
-        <v>Cash Withdrawal</v>
-      </c>
-      <c r="C50" t="str">
+      <c r="B51" t="str">
+        <v>Cash Withdrawal</v>
+      </c>
+      <c r="C51" t="str">
         <v>TT2324100671</v>
       </c>
-      <c r="D50" t="str">
+      <c r="D51" t="str">
         <v>29/08/2023</v>
       </c>
-      <c r="E50">
+      <c r="E51">
         <v>72041.59</v>
       </c>
-      <c r="G50">
+      <c r="G51">
         <v>2866283.38</v>
       </c>
     </row>
-    <row r="51" xml:space="preserve">
-      <c r="A51" t="str">
+    <row r="52" xml:space="preserve">
+      <c r="A52" t="str">
         <v>07/09/2023</v>
       </c>
-      <c r="B51" t="str" xml:space="preserve">
+      <c r="B52" t="str" xml:space="preserve">
         <v xml:space="preserve">Cash Withdrawal_x000d_
 WDR MABEL AKO ABANG IFO SAMUEL SAKA BOATENG AND OTHER</v>
       </c>
-      <c r="C51" t="str">
+      <c r="C52" t="str">
         <v>TT2325000414</v>
-      </c>
-      <c r="D51" t="str">
-        <v/>
-      </c>
-      <c r="E51">
-        <v>97691.61</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="str">
-        <v>07/09/2023</v>
-      </c>
-      <c r="B52" t="str">
-        <v>Cash Withdrawal WDR MABEL AKO-ABANG</v>
-      </c>
-      <c r="C52" t="str">
-        <v>TT2325000584</v>
       </c>
       <c r="D52" t="str">
         <v/>
       </c>
       <c r="E52">
-        <v>127761.84</v>
+        <v>97691.61</v>
+      </c>
+      <c r="G52">
+        <v>2768591.77</v>
       </c>
     </row>
     <row r="53">
@@ -1264,16 +1345,19 @@
         <v>07/09/2023</v>
       </c>
       <c r="B53" t="str">
-        <v>Cash Withdrawal WDR MABEL AKO ABANG IFO REV EDWIN AFARI</v>
+        <v>Cash Withdrawal WDR MABEL AKO-ABANG</v>
       </c>
       <c r="C53" t="str">
-        <v>TT2325000606</v>
+        <v>TT2325000584</v>
       </c>
       <c r="D53" t="str">
         <v/>
       </c>
       <c r="E53">
-        <v>16557.9</v>
+        <v>127761.84</v>
+      </c>
+      <c r="G53">
+        <v>2640829.93</v>
       </c>
     </row>
     <row r="54">
@@ -1281,38 +1365,64 @@
         <v>07/09/2023</v>
       </c>
       <c r="B54" t="str">
-        <v>Cash Withdrawal WDR MABEL AKO ABANG IFO FRANCIS NANA YAW CODJO AND OTHERS</v>
+        <v>Cash Withdrawal WDR MABEL AKO ABANG IFO REV EDWIN AFARI</v>
       </c>
       <c r="C54" t="str">
-        <v>TT2325000598</v>
+        <v>TT2325000606</v>
       </c>
       <c r="D54" t="str">
         <v/>
       </c>
       <c r="E54">
-        <v>19869.48</v>
+        <v>16557.9</v>
+      </c>
+      <c r="G54">
+        <v>2624272.03</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>29/09/2023</v>
+        <v>07/09/2023</v>
       </c>
       <c r="B55" t="str">
-        <v>Cash Withdrawal WDR AKO-ABANG MABEL IFO PETER MAC MANU AND OTHERS</v>
+        <v>Cash Withdrawal WDR MABEL AKO ABANG IFO FRANCIS NANA YAW CODJO AND OTHERS</v>
       </c>
       <c r="C55" t="str">
-        <v>TT2327200618</v>
+        <v>TT2325000598</v>
       </c>
       <c r="D55" t="str">
         <v/>
       </c>
       <c r="E55">
+        <v>19869.48</v>
+      </c>
+      <c r="G55">
+        <v>2604402.55</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>29/09/2023</v>
+      </c>
+      <c r="B56" t="str">
+        <v>Cash Withdrawal WDR AKO-ABANG MABEL IFO PETER MAC MANU AND OTHERS</v>
+      </c>
+      <c r="C56" t="str">
+        <v>TT2327200618</v>
+      </c>
+      <c r="D56" t="str">
+        <v/>
+      </c>
+      <c r="E56">
         <v>363414.72</v>
+      </c>
+      <c r="G56">
+        <v>2240987.83</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G55"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G56"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>